<commit_message>
Actualiza leads: Balmoral, Casa Bianca, Clayton, Antigua, Royal Pacific, Terranova y corrige duplicado
</commit_message>
<xml_diff>
--- a/AniCare_Sistema_Leads_Panama.xlsx
+++ b/AniCare_Sistema_Leads_Panama.xlsx
@@ -14,9 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VISITADOS" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leads'!$A$1:$O$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Leads'!$A$1:$O$164</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Leads'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Leads'!$A$1:$O$134</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Leads'!$A$1:$O$164</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Resumen'!$A$1:$B$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1025,7 +1025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O134"/>
+  <dimension ref="A1:O163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8105,15 +8105,40 @@
         <f>IF(B121="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B121" s="7" t="n"/>
-      <c r="C121" s="7" t="n"/>
-      <c r="D121" s="7" t="n"/>
-      <c r="E121" s="7" t="n"/>
-      <c r="F121" s="7" t="n"/>
-      <c r="G121" s="7" t="n"/>
-      <c r="H121" s="7" t="n"/>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>Balmoral Gardens</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>Pedregal</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>Calle 1ra Oeste, Urb. Balmoral, Pedregal, Panamá</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr"/>
+      <c r="G121" s="7" t="inlineStr"/>
+      <c r="H121" s="7" t="inlineStr"/>
       <c r="I121" s="7" t="n"/>
-      <c r="K121" s="7" t="n"/>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K121" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L121" s="8">
         <f>IF(B121="","",IF(COUNTIFS($B$2:B121,B121,$D$2:D121,D121)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8126,22 +8151,51 @@
         <f>IF(F121="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F121,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O121" s="7" t="n"/>
+      <c r="O121" s="7" t="inlineStr">
+        <is>
+          <t>Proyecto de BAU Panamá / Balmoral Gardens S.A. Sin teléfono de administración público — solo formulario de contacto de ventas en baupanama.com. Verificar en persona.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="6">
         <f>IF(B122="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B122" s="7" t="n"/>
-      <c r="C122" s="7" t="n"/>
-      <c r="D122" s="7" t="n"/>
-      <c r="E122" s="7" t="n"/>
-      <c r="F122" s="7" t="n"/>
-      <c r="G122" s="7" t="n"/>
-      <c r="H122" s="7" t="n"/>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t>PH Terrazas del Balmoral</t>
+        </is>
+      </c>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t>Pedregal</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>Vía C. Rana de Oro, Pedregal, Panamá</t>
+        </is>
+      </c>
+      <c r="F122" s="7" t="inlineStr"/>
+      <c r="G122" s="7" t="inlineStr"/>
+      <c r="H122" s="7" t="inlineStr"/>
       <c r="I122" s="7" t="n"/>
-      <c r="K122" s="7" t="n"/>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K122" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L122" s="8">
         <f>IF(B122="","",IF(COUNTIFS($B$2:B122,B122,$D$2:D122,D122)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8154,22 +8208,51 @@
         <f>IF(F122="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F122,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O122" s="7" t="n"/>
+      <c r="O122" s="7" t="inlineStr">
+        <is>
+          <t>Confirmado en listados inmobiliarios (Remax, Casa Solution). Sin teléfono de administración público — verificar en persona.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="6">
         <f>IF(B123="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B123" s="7" t="n"/>
-      <c r="C123" s="7" t="n"/>
-      <c r="D123" s="7" t="n"/>
-      <c r="E123" s="7" t="n"/>
-      <c r="F123" s="7" t="n"/>
-      <c r="G123" s="7" t="n"/>
-      <c r="H123" s="7" t="n"/>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t>PH Balmoral</t>
+        </is>
+      </c>
+      <c r="C123" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="inlineStr">
+        <is>
+          <t>Pedregal</t>
+        </is>
+      </c>
+      <c r="E123" s="7" t="inlineStr">
+        <is>
+          <t>Urb. Balmoral, Pedregal, Panamá</t>
+        </is>
+      </c>
+      <c r="F123" s="7" t="inlineStr"/>
+      <c r="G123" s="7" t="inlineStr"/>
+      <c r="H123" s="7" t="inlineStr"/>
       <c r="I123" s="7" t="n"/>
-      <c r="K123" s="7" t="n"/>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K123" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L123" s="8">
         <f>IF(B123="","",IF(COUNTIFS($B$2:B123,B123,$D$2:D123,D123)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8182,22 +8265,51 @@
         <f>IF(F123="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F123,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O123" s="7" t="n"/>
+      <c r="O123" s="7" t="inlineStr">
+        <is>
+          <t>Nombre genérico de la urbanización Balmoral — podría referirse al mismo complejo que Balmoral Gardens o Terrazas del Balmoral. Confirmar en el lugar cuál PH específico es. Sin teléfono público.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="6">
         <f>IF(B124="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B124" s="7" t="n"/>
-      <c r="C124" s="7" t="n"/>
-      <c r="D124" s="7" t="n"/>
-      <c r="E124" s="7" t="n"/>
-      <c r="F124" s="7" t="n"/>
-      <c r="G124" s="7" t="n"/>
-      <c r="H124" s="7" t="n"/>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>Urbanización Balmoral</t>
+        </is>
+      </c>
+      <c r="C124" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="inlineStr">
+        <is>
+          <t>Pedregal</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="inlineStr">
+        <is>
+          <t>Av. Paseo del Mar, Urb. Balmoral, Pedregal, Panamá</t>
+        </is>
+      </c>
+      <c r="F124" s="7" t="inlineStr"/>
+      <c r="G124" s="7" t="inlineStr"/>
+      <c r="H124" s="7" t="inlineStr"/>
       <c r="I124" s="7" t="n"/>
-      <c r="K124" s="7" t="n"/>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K124" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L124" s="8">
         <f>IF(B124="","",IF(COUNTIFS($B$2:B124,B124,$D$2:D124,D124)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8210,7 +8322,11 @@
         <f>IF(F124="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F124,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O124" s="7" t="n"/>
+      <c r="O124" s="7" t="inlineStr">
+        <is>
+          <t>Urbanización completa (varios edificios/PH adentro). Sin teléfono de administración general público — verificar en persona.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="6">
@@ -8274,15 +8390,40 @@
         <f>IF(B126="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B126" s="7" t="n"/>
-      <c r="C126" s="7" t="n"/>
-      <c r="D126" s="7" t="n"/>
-      <c r="E126" s="7" t="n"/>
-      <c r="F126" s="7" t="n"/>
-      <c r="G126" s="7" t="n"/>
-      <c r="H126" s="7" t="n"/>
+      <c r="B126" s="7" t="inlineStr">
+        <is>
+          <t>Residencial Balmoral</t>
+        </is>
+      </c>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="inlineStr">
+        <is>
+          <t>Costa del Este</t>
+        </is>
+      </c>
+      <c r="E126" s="7" t="inlineStr">
+        <is>
+          <t>Costa del Este, Panamá (dirección exacta no confirmada)</t>
+        </is>
+      </c>
+      <c r="F126" s="7" t="inlineStr"/>
+      <c r="G126" s="7" t="inlineStr"/>
+      <c r="H126" s="7" t="inlineStr"/>
       <c r="I126" s="7" t="n"/>
-      <c r="K126" s="7" t="n"/>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K126" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L126" s="8">
         <f>IF(B126="","",IF(COUNTIFS($B$2:B126,B126,$D$2:D126,D126)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8295,22 +8436,63 @@
         <f>IF(F126="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F126,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O126" s="7" t="n"/>
+      <c r="O126" s="7" t="inlineStr">
+        <is>
+          <t>Portales inmobiliarios lo listan como 'Balmoral - Costa del Este', distinto de la urbanización Balmoral en Pedregal — podría haber confusión de nombres entre ambos. Confirmar cuál es antes de visitar. Sin teléfono público.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="6">
         <f>IF(B127="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B127" s="7" t="n"/>
-      <c r="C127" s="7" t="n"/>
-      <c r="D127" s="7" t="n"/>
-      <c r="E127" s="7" t="n"/>
-      <c r="F127" s="7" t="n"/>
-      <c r="G127" s="7" t="n"/>
-      <c r="H127" s="7" t="n"/>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
+          <t>Casa Bianca</t>
+        </is>
+      </c>
+      <c r="C127" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="inlineStr">
+        <is>
+          <t>Costa del Este</t>
+        </is>
+      </c>
+      <c r="E127" s="7" t="inlineStr">
+        <is>
+          <t>Ave. Paseo del Mar, frente a Town Center, Costa del Este, Panamá</t>
+        </is>
+      </c>
+      <c r="F127" s="7" t="inlineStr">
+        <is>
+          <t>214-2376</t>
+        </is>
+      </c>
+      <c r="G127" s="7" t="inlineStr">
+        <is>
+          <t>administracion@empresasbern.com</t>
+        </is>
+      </c>
+      <c r="H127" s="7" t="inlineStr">
+        <is>
+          <t>empresasbern.com</t>
+        </is>
+      </c>
       <c r="I127" s="7" t="n"/>
-      <c r="K127" s="7" t="n"/>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K127" s="7" t="inlineStr">
+        <is>
+          <t>Verificado por teléfono</t>
+        </is>
+      </c>
       <c r="L127" s="8">
         <f>IF(B127="","",IF(COUNTIFS($B$2:B127,B127,$D$2:D127,D127)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8323,22 +8505,51 @@
         <f>IF(F127="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F127,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O127" s="7" t="n"/>
+      <c r="O127" s="7" t="inlineStr">
+        <is>
+          <t>Confirmado — proyecto de Empresas Bern. Teléfono y correo de administración públicos y verificados.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="6">
         <f>IF(B128="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B128" s="7" t="n"/>
-      <c r="C128" s="7" t="n"/>
-      <c r="D128" s="7" t="n"/>
-      <c r="E128" s="7" t="n"/>
-      <c r="F128" s="7" t="n"/>
-      <c r="G128" s="7" t="n"/>
-      <c r="H128" s="7" t="n"/>
+      <c r="B128" s="7" t="inlineStr">
+        <is>
+          <t>PH Casa Bella</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="inlineStr">
+        <is>
+          <t>Parque Lefevre</t>
+        </is>
+      </c>
+      <c r="E128" s="7" t="inlineStr">
+        <is>
+          <t>Calle María Herrera, Parque Lefevre, Panamá</t>
+        </is>
+      </c>
+      <c r="F128" s="7" t="inlineStr"/>
+      <c r="G128" s="7" t="inlineStr"/>
+      <c r="H128" s="7" t="inlineStr"/>
       <c r="I128" s="7" t="n"/>
-      <c r="K128" s="7" t="n"/>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K128" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L128" s="8">
         <f>IF(B128="","",IF(COUNTIFS($B$2:B128,B128,$D$2:D128,D128)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8351,22 +8562,51 @@
         <f>IF(F128="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F128,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O128" s="7" t="n"/>
+      <c r="O128" s="7" t="inlineStr">
+        <is>
+          <t>No se encontró registro público (web) de este PH con ese nombre y dirección — dato aportado directamente por Ani. Verificar en persona, sin fuente online que lo confirme.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="6">
         <f>IF(B129="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B129" s="7" t="n"/>
-      <c r="C129" s="7" t="n"/>
-      <c r="D129" s="7" t="n"/>
-      <c r="E129" s="7" t="n"/>
-      <c r="F129" s="7" t="n"/>
-      <c r="G129" s="7" t="n"/>
-      <c r="H129" s="7" t="n"/>
+      <c r="B129" s="7" t="inlineStr">
+        <is>
+          <t>Casablanca</t>
+        </is>
+      </c>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D129" s="7" t="inlineStr">
+        <is>
+          <t>Santa María</t>
+        </is>
+      </c>
+      <c r="E129" s="7" t="inlineStr">
+        <is>
+          <t>Santa María, Costa del Este, Panamá (dirección exacta no confirmada)</t>
+        </is>
+      </c>
+      <c r="F129" s="7" t="inlineStr"/>
+      <c r="G129" s="7" t="inlineStr"/>
+      <c r="H129" s="7" t="inlineStr"/>
       <c r="I129" s="7" t="n"/>
-      <c r="K129" s="7" t="n"/>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K129" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L129" s="8">
         <f>IF(B129="","",IF(COUNTIFS($B$2:B129,B129,$D$2:D129,D129)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8379,22 +8619,51 @@
         <f>IF(F129="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F129,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O129" s="7" t="n"/>
+      <c r="O129" s="7" t="inlineStr">
+        <is>
+          <t>No se encontró un PH residencial con ese nombre en Santa María — la búsqueda solo devolvió un restaurante y un distrito de negocios de nombre similar en Casco Viejo. Verificar en persona.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="6">
         <f>IF(B130="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B130" s="7" t="n"/>
-      <c r="C130" s="7" t="n"/>
-      <c r="D130" s="7" t="n"/>
-      <c r="E130" s="7" t="n"/>
-      <c r="F130" s="7" t="n"/>
-      <c r="G130" s="7" t="n"/>
-      <c r="H130" s="7" t="n"/>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>Residencial Antigua</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t>Costa del Este</t>
+        </is>
+      </c>
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>Av. Marina del Norte, Costa del Este, Panamá</t>
+        </is>
+      </c>
+      <c r="F130" s="7" t="inlineStr"/>
+      <c r="G130" s="7" t="inlineStr"/>
+      <c r="H130" s="7" t="inlineStr"/>
       <c r="I130" s="7" t="n"/>
-      <c r="K130" s="7" t="n"/>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K130" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L130" s="8">
         <f>IF(B130="","",IF(COUNTIFS($B$2:B130,B130,$D$2:D130,D130)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8407,22 +8676,51 @@
         <f>IF(F130="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F130,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O130" s="7" t="n"/>
+      <c r="O130" s="7" t="inlineStr">
+        <is>
+          <t>Desarrollo residencial exclusivo con seguridad 24/7. Solo se encontró contacto de agencias inmobiliarias que venden ahí, no de la administración del PH. Verificar en persona.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="6">
         <f>IF(B131="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B131" s="7" t="n"/>
-      <c r="C131" s="7" t="n"/>
-      <c r="D131" s="7" t="n"/>
-      <c r="E131" s="7" t="n"/>
-      <c r="F131" s="7" t="n"/>
-      <c r="G131" s="7" t="n"/>
-      <c r="H131" s="7" t="n"/>
+      <c r="B131" s="7" t="inlineStr">
+        <is>
+          <t>Residencial Royal Pacific</t>
+        </is>
+      </c>
+      <c r="C131" s="7" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="inlineStr">
+        <is>
+          <t>Costa del Este</t>
+        </is>
+      </c>
+      <c r="E131" s="7" t="inlineStr">
+        <is>
+          <t>Costa del Este (Juan Díaz), Panamá</t>
+        </is>
+      </c>
+      <c r="F131" s="7" t="inlineStr"/>
+      <c r="G131" s="7" t="inlineStr"/>
+      <c r="H131" s="7" t="inlineStr"/>
       <c r="I131" s="7" t="n"/>
-      <c r="K131" s="7" t="n"/>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K131" s="7" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
       <c r="L131" s="8">
         <f>IF(B131="","",IF(COUNTIFS($B$2:B131,B131,$D$2:D131,D131)&gt;1,"SI","NO"))</f>
         <v/>
@@ -8435,17 +8733,99 @@
         <f>IF(F131="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F131,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
         <v/>
       </c>
-      <c r="O131" s="7" t="n"/>
+      <c r="O131" s="7" t="inlineStr">
+        <is>
+          <t>Ojo: existe otro 'Royal Pacific' distinto en Punta Pacífica/San Francisco (torre de 24 pisos) — no confundir. Este es el de Costa del Este/Juan Díaz. Sin teléfono de administración público, solo contacto de agencia inmobiliaria (Grupo Tribaldos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>PH Terranova</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>El Cangrejo</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Calle Enrique Greenzier, El Cangrejo, Panamá</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>Torre de 25 pisos, construida en 2000. Sin teléfono de administración público, solo contactos de agencias inmobiliarias (Padeco Realty, Alpha Group).</t>
+        </is>
+      </c>
     </row>
     <row r="133">
-      <c r="B133" s="9" t="inlineStr">
-        <is>
-          <t>Leyenda: celdas amarillas = tú las llenas a mano. Columnas K, L, M se calculan solas. No edites la columna ID ni K/L/M.</t>
+      <c r="A133">
+        <f>IF(B133="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>PH Clayton Park I</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Clayton</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Clayton (Corregimiento Ancón), Panamá</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
+      <c r="L133">
+        <f>IF(B133="","",IF(COUNTIFS($B$2:B133,B133,$D$2:D133,D133)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M133">
+        <f>IF(G133="","",IF(AND(ISNUMBER(SEARCH("@",G133)),ISNUMBER(SEARCH(".",G133,SEARCH("@",G133))),LEN(G133)-LEN(SUBSTITUTE(G133,"@",""))=1,MID(G133,SEARCH("@",G133)+1,1)&lt;&gt;".",RIGHT(G133,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N133">
+        <f>IF(F133="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F133,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>Comunidad residencial en Clayton. Sin teléfono de administración público — verificar en persona.</t>
         </is>
       </c>
     </row>
@@ -8456,7 +8836,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>P.H. Mirador del Golf</t>
+          <t>PH Clayton Park II</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -8466,12 +8846,22 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Parque Lefevre</t>
+          <t>Clayton</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Calle 1era, Parque Lefevre, Ciudad de Panamá</t>
+          <t>Calle al Hospital, Clayton, Panamá</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>304-9830 / 301-0083</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>gproviviendan.com</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -8481,17 +8871,685 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Por verificar</t>
-        </is>
+          <t>Verificado por teléfono</t>
+        </is>
+      </c>
+      <c r="L134">
+        <f>IF(B134="","",IF(COUNTIFS($B$2:B134,B134,$D$2:D134,D134)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M134">
+        <f>IF(G134="","",IF(AND(ISNUMBER(SEARCH("@",G134)),ISNUMBER(SEARCH(".",G134,SEARCH("@",G134))),LEN(G134)-LEN(SUBSTITUTE(G134,"@",""))=1,MID(G134,SEARCH("@",G134)+1,1)&lt;&gt;".",RIGHT(G134,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N134">
+        <f>IF(F134="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F134,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>Torre de 12 pisos (2012), cerca de Parque Omar. Sin teléfono público listado — verificar en portería o con la administración en persona.</t>
+          <t>Confirmado — desarrollo de Grupo Provivienda. 3 torres de 17 pisos. 304-9830 = oficina administrativa, 301-0083 = oficina de ventas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135">
+        <f>IF(B135="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Clayton Tower</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Clayton</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Clayton (Corregimiento Ancón), Panamá</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
+      <c r="L135">
+        <f>IF(B135="","",IF(COUNTIFS($B$2:B135,B135,$D$2:D135,D135)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M135">
+        <f>IF(G135="","",IF(AND(ISNUMBER(SEARCH("@",G135)),ISNUMBER(SEARCH(".",G135,SEARCH("@",G135))),LEN(G135)-LEN(SUBSTITUTE(G135,"@",""))=1,MID(G135,SEARCH("@",G135)+1,1)&lt;&gt;".",RIGHT(G135,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N135">
+        <f>IF(F135="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F135,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>Mencionado en listados inmobiliarios de la zona, información muy escasa. Sin dirección exacta ni teléfono confirmados — verificar en persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136">
+        <f>IF(B136="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Clayton Village</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Clayton</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Clayton (Corregimiento Ancón), Panamá</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
+      <c r="L136">
+        <f>IF(B136="","",IF(COUNTIFS($B$2:B136,B136,$D$2:D136,D136)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M136">
+        <f>IF(G136="","",IF(AND(ISNUMBER(SEARCH("@",G136)),ISNUMBER(SEARCH(".",G136,SEARCH("@",G136))),LEN(G136)-LEN(SUBSTITUTE(G136,"@",""))=1,MID(G136,SEARCH("@",G136)+1,1)&lt;&gt;".",RIGHT(G136,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N136">
+        <f>IF(F136="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F136,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>Comunidad residencial cerrada con seguridad 24h. Sin teléfono de administración público — verificar en persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137">
+        <f>IF(B137="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Residencial Veranda</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Costa del Este</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Calle R.36, Costa del Este, Panamá</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
+      <c r="L137">
+        <f>IF(B137="","",IF(COUNTIFS($B$2:B137,B137,$D$2:D137,D137)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M137">
+        <f>IF(G137="","",IF(AND(ISNUMBER(SEARCH("@",G137)),ISNUMBER(SEARCH(".",G137,SEARCH("@",G137))),LEN(G137)-LEN(SUBSTITUTE(G137,"@",""))=1,MID(G137,SEARCH("@",G137)+1,1)&lt;&gt;".",RIGHT(G137,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N137">
+        <f>IF(F137="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F137,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>Confirmado como desarrollo en Costa del Este. Sin teléfono de administración público, solo agencias inmobiliarias — verificar en persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138">
+        <f>IF(B138="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Residencial Costa Azul</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>PH/Residencial</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Costa del Este</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Costa del Este, Panamá</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Sin verificar</t>
+        </is>
+      </c>
+      <c r="L138">
+        <f>IF(B138="","",IF(COUNTIFS($B$2:B138,B138,$D$2:D138,D138)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M138">
+        <f>IF(G138="","",IF(AND(ISNUMBER(SEARCH("@",G138)),ISNUMBER(SEARCH(".",G138,SEARCH("@",G138))),LEN(G138)-LEN(SUBSTITUTE(G138,"@",""))=1,MID(G138,SEARCH("@",G138)+1,1)&lt;&gt;".",RIGHT(G138,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N138">
+        <f>IF(F138="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F138,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>Residencial con seguridad 24/7 en el corazón de Costa del Este. Sin teléfono de administración público, solo agencias inmobiliarias — verificar en persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139">
+        <f>IF(B139="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L139">
+        <f>IF(B139="","",IF(COUNTIFS($B$2:B139,B139,$D$2:D139,D139)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M139">
+        <f>IF(G139="","",IF(AND(ISNUMBER(SEARCH("@",G139)),ISNUMBER(SEARCH(".",G139,SEARCH("@",G139))),LEN(G139)-LEN(SUBSTITUTE(G139,"@",""))=1,MID(G139,SEARCH("@",G139)+1,1)&lt;&gt;".",RIGHT(G139,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N139">
+        <f>IF(F139="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F139,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140">
+        <f>IF(B140="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L140">
+        <f>IF(B140="","",IF(COUNTIFS($B$2:B140,B140,$D$2:D140,D140)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M140">
+        <f>IF(G140="","",IF(AND(ISNUMBER(SEARCH("@",G140)),ISNUMBER(SEARCH(".",G140,SEARCH("@",G140))),LEN(G140)-LEN(SUBSTITUTE(G140,"@",""))=1,MID(G140,SEARCH("@",G140)+1,1)&lt;&gt;".",RIGHT(G140,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N140">
+        <f>IF(F140="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F140,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141">
+        <f>IF(B141="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L141">
+        <f>IF(B141="","",IF(COUNTIFS($B$2:B141,B141,$D$2:D141,D141)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M141">
+        <f>IF(G141="","",IF(AND(ISNUMBER(SEARCH("@",G141)),ISNUMBER(SEARCH(".",G141,SEARCH("@",G141))),LEN(G141)-LEN(SUBSTITUTE(G141,"@",""))=1,MID(G141,SEARCH("@",G141)+1,1)&lt;&gt;".",RIGHT(G141,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N141">
+        <f>IF(F141="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F141,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142">
+        <f>IF(B142="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L142">
+        <f>IF(B142="","",IF(COUNTIFS($B$2:B142,B142,$D$2:D142,D142)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M142">
+        <f>IF(G142="","",IF(AND(ISNUMBER(SEARCH("@",G142)),ISNUMBER(SEARCH(".",G142,SEARCH("@",G142))),LEN(G142)-LEN(SUBSTITUTE(G142,"@",""))=1,MID(G142,SEARCH("@",G142)+1,1)&lt;&gt;".",RIGHT(G142,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N142">
+        <f>IF(F142="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F142,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143">
+        <f>IF(B143="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L143">
+        <f>IF(B143="","",IF(COUNTIFS($B$2:B143,B143,$D$2:D143,D143)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M143">
+        <f>IF(G143="","",IF(AND(ISNUMBER(SEARCH("@",G143)),ISNUMBER(SEARCH(".",G143,SEARCH("@",G143))),LEN(G143)-LEN(SUBSTITUTE(G143,"@",""))=1,MID(G143,SEARCH("@",G143)+1,1)&lt;&gt;".",RIGHT(G143,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N143">
+        <f>IF(F143="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F143,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144">
+        <f>IF(B144="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L144">
+        <f>IF(B144="","",IF(COUNTIFS($B$2:B144,B144,$D$2:D144,D144)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M144">
+        <f>IF(G144="","",IF(AND(ISNUMBER(SEARCH("@",G144)),ISNUMBER(SEARCH(".",G144,SEARCH("@",G144))),LEN(G144)-LEN(SUBSTITUTE(G144,"@",""))=1,MID(G144,SEARCH("@",G144)+1,1)&lt;&gt;".",RIGHT(G144,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N144">
+        <f>IF(F144="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F144,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145">
+        <f>IF(B145="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L145">
+        <f>IF(B145="","",IF(COUNTIFS($B$2:B145,B145,$D$2:D145,D145)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M145">
+        <f>IF(G145="","",IF(AND(ISNUMBER(SEARCH("@",G145)),ISNUMBER(SEARCH(".",G145,SEARCH("@",G145))),LEN(G145)-LEN(SUBSTITUTE(G145,"@",""))=1,MID(G145,SEARCH("@",G145)+1,1)&lt;&gt;".",RIGHT(G145,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N145">
+        <f>IF(F145="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F145,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146">
+        <f>IF(B146="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L146">
+        <f>IF(B146="","",IF(COUNTIFS($B$2:B146,B146,$D$2:D146,D146)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M146">
+        <f>IF(G146="","",IF(AND(ISNUMBER(SEARCH("@",G146)),ISNUMBER(SEARCH(".",G146,SEARCH("@",G146))),LEN(G146)-LEN(SUBSTITUTE(G146,"@",""))=1,MID(G146,SEARCH("@",G146)+1,1)&lt;&gt;".",RIGHT(G146,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N146">
+        <f>IF(F146="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F146,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147">
+        <f>IF(B147="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L147">
+        <f>IF(B147="","",IF(COUNTIFS($B$2:B147,B147,$D$2:D147,D147)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M147">
+        <f>IF(G147="","",IF(AND(ISNUMBER(SEARCH("@",G147)),ISNUMBER(SEARCH(".",G147,SEARCH("@",G147))),LEN(G147)-LEN(SUBSTITUTE(G147,"@",""))=1,MID(G147,SEARCH("@",G147)+1,1)&lt;&gt;".",RIGHT(G147,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N147">
+        <f>IF(F147="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F147,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148">
+        <f>IF(B148="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L148">
+        <f>IF(B148="","",IF(COUNTIFS($B$2:B148,B148,$D$2:D148,D148)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M148">
+        <f>IF(G148="","",IF(AND(ISNUMBER(SEARCH("@",G148)),ISNUMBER(SEARCH(".",G148,SEARCH("@",G148))),LEN(G148)-LEN(SUBSTITUTE(G148,"@",""))=1,MID(G148,SEARCH("@",G148)+1,1)&lt;&gt;".",RIGHT(G148,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N148">
+        <f>IF(F148="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F148,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149">
+        <f>IF(B149="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L149">
+        <f>IF(B149="","",IF(COUNTIFS($B$2:B149,B149,$D$2:D149,D149)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M149">
+        <f>IF(G149="","",IF(AND(ISNUMBER(SEARCH("@",G149)),ISNUMBER(SEARCH(".",G149,SEARCH("@",G149))),LEN(G149)-LEN(SUBSTITUTE(G149,"@",""))=1,MID(G149,SEARCH("@",G149)+1,1)&lt;&gt;".",RIGHT(G149,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N149">
+        <f>IF(F149="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F149,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150">
+        <f>IF(B150="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L150">
+        <f>IF(B150="","",IF(COUNTIFS($B$2:B150,B150,$D$2:D150,D150)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M150">
+        <f>IF(G150="","",IF(AND(ISNUMBER(SEARCH("@",G150)),ISNUMBER(SEARCH(".",G150,SEARCH("@",G150))),LEN(G150)-LEN(SUBSTITUTE(G150,"@",""))=1,MID(G150,SEARCH("@",G150)+1,1)&lt;&gt;".",RIGHT(G150,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N150">
+        <f>IF(F150="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F150,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151">
+        <f>IF(B151="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L151">
+        <f>IF(B151="","",IF(COUNTIFS($B$2:B151,B151,$D$2:D151,D151)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M151">
+        <f>IF(G151="","",IF(AND(ISNUMBER(SEARCH("@",G151)),ISNUMBER(SEARCH(".",G151,SEARCH("@",G151))),LEN(G151)-LEN(SUBSTITUTE(G151,"@",""))=1,MID(G151,SEARCH("@",G151)+1,1)&lt;&gt;".",RIGHT(G151,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N151">
+        <f>IF(F151="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F151,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152">
+        <f>IF(B152="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L152">
+        <f>IF(B152="","",IF(COUNTIFS($B$2:B152,B152,$D$2:D152,D152)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M152">
+        <f>IF(G152="","",IF(AND(ISNUMBER(SEARCH("@",G152)),ISNUMBER(SEARCH(".",G152,SEARCH("@",G152))),LEN(G152)-LEN(SUBSTITUTE(G152,"@",""))=1,MID(G152,SEARCH("@",G152)+1,1)&lt;&gt;".",RIGHT(G152,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N152">
+        <f>IF(F152="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F152,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153">
+        <f>IF(B153="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L153">
+        <f>IF(B153="","",IF(COUNTIFS($B$2:B153,B153,$D$2:D153,D153)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M153">
+        <f>IF(G153="","",IF(AND(ISNUMBER(SEARCH("@",G153)),ISNUMBER(SEARCH(".",G153,SEARCH("@",G153))),LEN(G153)-LEN(SUBSTITUTE(G153,"@",""))=1,MID(G153,SEARCH("@",G153)+1,1)&lt;&gt;".",RIGHT(G153,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N153">
+        <f>IF(F153="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F153,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154">
+        <f>IF(B154="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L154">
+        <f>IF(B154="","",IF(COUNTIFS($B$2:B154,B154,$D$2:D154,D154)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M154">
+        <f>IF(G154="","",IF(AND(ISNUMBER(SEARCH("@",G154)),ISNUMBER(SEARCH(".",G154,SEARCH("@",G154))),LEN(G154)-LEN(SUBSTITUTE(G154,"@",""))=1,MID(G154,SEARCH("@",G154)+1,1)&lt;&gt;".",RIGHT(G154,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N154">
+        <f>IF(F154="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F154,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155">
+        <f>IF(B155="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L155">
+        <f>IF(B155="","",IF(COUNTIFS($B$2:B155,B155,$D$2:D155,D155)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M155">
+        <f>IF(G155="","",IF(AND(ISNUMBER(SEARCH("@",G155)),ISNUMBER(SEARCH(".",G155,SEARCH("@",G155))),LEN(G155)-LEN(SUBSTITUTE(G155,"@",""))=1,MID(G155,SEARCH("@",G155)+1,1)&lt;&gt;".",RIGHT(G155,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N155">
+        <f>IF(F155="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F155,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156">
+        <f>IF(B156="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L156">
+        <f>IF(B156="","",IF(COUNTIFS($B$2:B156,B156,$D$2:D156,D156)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M156">
+        <f>IF(G156="","",IF(AND(ISNUMBER(SEARCH("@",G156)),ISNUMBER(SEARCH(".",G156,SEARCH("@",G156))),LEN(G156)-LEN(SUBSTITUTE(G156,"@",""))=1,MID(G156,SEARCH("@",G156)+1,1)&lt;&gt;".",RIGHT(G156,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N156">
+        <f>IF(F156="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F156,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157">
+        <f>IF(B157="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L157">
+        <f>IF(B157="","",IF(COUNTIFS($B$2:B157,B157,$D$2:D157,D157)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M157">
+        <f>IF(G157="","",IF(AND(ISNUMBER(SEARCH("@",G157)),ISNUMBER(SEARCH(".",G157,SEARCH("@",G157))),LEN(G157)-LEN(SUBSTITUTE(G157,"@",""))=1,MID(G157,SEARCH("@",G157)+1,1)&lt;&gt;".",RIGHT(G157,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N157">
+        <f>IF(F157="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F157,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158">
+        <f>IF(B158="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L158">
+        <f>IF(B158="","",IF(COUNTIFS($B$2:B158,B158,$D$2:D158,D158)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M158">
+        <f>IF(G158="","",IF(AND(ISNUMBER(SEARCH("@",G158)),ISNUMBER(SEARCH(".",G158,SEARCH("@",G158))),LEN(G158)-LEN(SUBSTITUTE(G158,"@",""))=1,MID(G158,SEARCH("@",G158)+1,1)&lt;&gt;".",RIGHT(G158,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N158">
+        <f>IF(F158="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F158,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159">
+        <f>IF(B159="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L159">
+        <f>IF(B159="","",IF(COUNTIFS($B$2:B159,B159,$D$2:D159,D159)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M159">
+        <f>IF(G159="","",IF(AND(ISNUMBER(SEARCH("@",G159)),ISNUMBER(SEARCH(".",G159,SEARCH("@",G159))),LEN(G159)-LEN(SUBSTITUTE(G159,"@",""))=1,MID(G159,SEARCH("@",G159)+1,1)&lt;&gt;".",RIGHT(G159,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N159">
+        <f>IF(F159="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F159,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160">
+        <f>IF(B160="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L160">
+        <f>IF(B160="","",IF(COUNTIFS($B$2:B160,B160,$D$2:D160,D160)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M160">
+        <f>IF(G160="","",IF(AND(ISNUMBER(SEARCH("@",G160)),ISNUMBER(SEARCH(".",G160,SEARCH("@",G160))),LEN(G160)-LEN(SUBSTITUTE(G160,"@",""))=1,MID(G160,SEARCH("@",G160)+1,1)&lt;&gt;".",RIGHT(G160,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N160">
+        <f>IF(F160="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F160,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161">
+        <f>IF(B161="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L161">
+        <f>IF(B161="","",IF(COUNTIFS($B$2:B161,B161,$D$2:D161,D161)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M161">
+        <f>IF(G161="","",IF(AND(ISNUMBER(SEARCH("@",G161)),ISNUMBER(SEARCH(".",G161,SEARCH("@",G161))),LEN(G161)-LEN(SUBSTITUTE(G161,"@",""))=1,MID(G161,SEARCH("@",G161)+1,1)&lt;&gt;".",RIGHT(G161,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N161">
+        <f>IF(F161="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F161,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162">
+        <f>IF(B162="","",ROW()-1)</f>
+        <v/>
+      </c>
+      <c r="L162">
+        <f>IF(B162="","",IF(COUNTIFS($B$2:B162,B162,$D$2:D162,D162)&gt;1,"SI","NO"))</f>
+        <v/>
+      </c>
+      <c r="M162">
+        <f>IF(G162="","",IF(AND(ISNUMBER(SEARCH("@",G162)),ISNUMBER(SEARCH(".",G162,SEARCH("@",G162))),LEN(G162)-LEN(SUBSTITUTE(G162,"@",""))=1,MID(G162,SEARCH("@",G162)+1,1)&lt;&gt;".",RIGHT(G162,1)&lt;&gt;"."),"Válido","Revisar"))</f>
+        <v/>
+      </c>
+      <c r="N162">
+        <f>IF(F162="","",IF(LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(F162,"+507",""),"-",""),"(",""),")",""))=8,"Válido","Revisar"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="B163" s="9" t="inlineStr">
+        <is>
+          <t>Leyenda: celdas amarillas = tú las llenas a mano. Columnas K, L, M se calculan solas. No edites la columna ID ni K/L/M.</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O134"/>
+  <autoFilter ref="A1:O164"/>
   <conditionalFormatting sqref="K2:K131">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"SI"</formula>
@@ -8517,16 +9575,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="C2:C134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Selecciona un valor de la lista" type="list">
+    <dataValidation sqref="C2:C164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Selecciona un valor de la lista" type="list">
       <formula1>"Hotel,PH/Residencial,Oficina,Clínica,Negocio general,Otro"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Selecciona un valor de la lista" type="list">
-      <formula1>"Costa del Este,Santa María,Versalles PH1,Reserva de Versalles,Versalles PH2,Don Bosco,Vía Brasil,Avenida Balboa,Punta Pacífica,Vía España,Condado del Rey,Obarrio / Bella Vista,Parque Lefevre,Marbella,Coco del Mar,San Francisco,El Cangrejo"</formula1>
+    <dataValidation sqref="D2:D164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Selecciona un valor de la lista" type="list">
+      <formula1>"Costa del Este,Santa María,Versalles PH1,Reserva de Versalles,Versalles PH2,Don Bosco,Vía Brasil,Avenida Balboa,Punta Pacífica,Vía España,Condado del Rey,Obarrio / Bella Vista,Parque Lefevre,Marbella,Coco del Mar,San Francisco,El Cangrejo,Pedregal,Clayton"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Selecciona un valor de la lista" type="list">
+    <dataValidation sqref="J2:J164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Selecciona un valor de la lista" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Selecciona un valor de la lista" type="list">
+    <dataValidation sqref="K2:K164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Entrada inválida" error="Selecciona un valor de la lista" type="list">
       <formula1>"Sin verificar,Verificado por teléfono,Verificado en persona,Contactado,No responde,Cliente"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8569,7 +9627,7 @@
         </is>
       </c>
       <c r="B4" s="13">
-        <f>COUNTA(Leads!B2:B134)-1</f>
+        <f>COUNTA(Leads!B2:B164)-1</f>
         <v/>
       </c>
     </row>
@@ -8580,7 +9638,7 @@
         </is>
       </c>
       <c r="B5" s="13">
-        <f>COUNTIF(Leads!L2:L134,"SI")</f>
+        <f>COUNTIF(Leads!L2:L164,"SI")</f>
         <v/>
       </c>
     </row>
@@ -8591,7 +9649,7 @@
         </is>
       </c>
       <c r="B6" s="13">
-        <f>COUNTIF(Leads!M2:M134,"Válido")</f>
+        <f>COUNTIF(Leads!M2:M164,"Válido")</f>
         <v/>
       </c>
     </row>
@@ -8602,7 +9660,7 @@
         </is>
       </c>
       <c r="B7" s="13">
-        <f>COUNTIF(Leads!N2:N134,"Válido")</f>
+        <f>COUNTIF(Leads!N2:N164,"Válido")</f>
         <v/>
       </c>
     </row>
@@ -8613,7 +9671,7 @@
         </is>
       </c>
       <c r="B8" s="13">
-        <f>COUNTIF(Leads!J2:J134,"Sí")</f>
+        <f>COUNTIF(Leads!J2:J164,"Sí")</f>
         <v/>
       </c>
     </row>

</xml_diff>